<commit_message>
Made changes on Propose Compensation page
</commit_message>
<xml_diff>
--- a/Data/Hires/testDataUS - Copy (2).xlsx
+++ b/Data/Hires/testDataUS - Copy (2).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F09EF8-AB4C-47BB-A407-3866FD404ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E65079C-5074-4FC4-9E49-45C364A4881E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="L2">
         <f t="shared" ref="L2:L17" ca="1" si="0">TODAY()-31</f>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M2" t="s">
         <v>56</v>
@@ -1288,13 +1288,13 @@
       <c r="W2" t="s">
         <v>62</v>
       </c>
-      <c r="X2">
+      <c r="X2" s="10">
         <f t="shared" ref="X2:X17" ca="1" si="1">L2</f>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y2">
         <f t="shared" ref="Y2:Y17" ca="1" si="2">TODAY()+20</f>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z2" t="s">
         <v>68</v>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="AR2">
         <f t="array" aca="1" ref="AR2:AR17" ca="1">_xlfn.RANDARRAY(16,1,123456789,999999999,FALSE)</f>
-        <v>278462587.30435622</v>
+        <v>728003728.51406848</v>
       </c>
       <c r="AS2" t="s">
         <v>82</v>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="L3">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M3" t="s">
         <v>56</v>
@@ -1459,13 +1459,13 @@
       <c r="W3" t="s">
         <v>62</v>
       </c>
-      <c r="X3">
+      <c r="X3" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y3">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z3" t="s">
         <v>68</v>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="AR3">
         <f ca="1"/>
-        <v>292832536.8641423</v>
+        <v>576759102.67173946</v>
       </c>
       <c r="AS3" t="s">
         <v>82</v>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L4">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M4" t="s">
         <v>56</v>
@@ -1630,13 +1630,13 @@
       <c r="W4" t="s">
         <v>62</v>
       </c>
-      <c r="X4">
+      <c r="X4" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y4">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z4" t="s">
         <v>68</v>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="AR4">
         <f ca="1"/>
-        <v>297172306.11195374</v>
+        <v>649243954.46533108</v>
       </c>
       <c r="AS4" t="s">
         <v>82</v>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="L5">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M5" t="s">
         <v>56</v>
@@ -1801,13 +1801,13 @@
       <c r="W5" t="s">
         <v>62</v>
       </c>
-      <c r="X5">
+      <c r="X5" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y5">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z5" t="s">
         <v>68</v>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="AR5">
         <f ca="1"/>
-        <v>427929662.90423727</v>
+        <v>635918102.95599687</v>
       </c>
       <c r="AS5" t="s">
         <v>82</v>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="L6">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M6" t="s">
         <v>56</v>
@@ -1972,13 +1972,13 @@
       <c r="W6" t="s">
         <v>62</v>
       </c>
-      <c r="X6">
+      <c r="X6" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y6">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z6" t="s">
         <v>68</v>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="AR6">
         <f ca="1"/>
-        <v>241081046.17868161</v>
+        <v>605113608.70800495</v>
       </c>
       <c r="AS6" t="s">
         <v>82</v>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="L7">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M7" t="s">
         <v>56</v>
@@ -2143,13 +2143,13 @@
       <c r="W7" t="s">
         <v>62</v>
       </c>
-      <c r="X7">
+      <c r="X7" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y7">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z7" t="s">
         <v>68</v>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="AR7">
         <f ca="1"/>
-        <v>209308476.63942516</v>
+        <v>659863402.47423196</v>
       </c>
       <c r="AS7" t="s">
         <v>82</v>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="L8">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M8" t="s">
         <v>56</v>
@@ -2314,13 +2314,13 @@
       <c r="W8" t="s">
         <v>62</v>
       </c>
-      <c r="X8">
+      <c r="X8" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y8">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z8" t="s">
         <v>68</v>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="AR8">
         <f ca="1"/>
-        <v>247702480.89073861</v>
+        <v>295605444.1000737</v>
       </c>
       <c r="AS8" t="s">
         <v>82</v>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="L9">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M9" t="s">
         <v>56</v>
@@ -2485,13 +2485,13 @@
       <c r="W9" t="s">
         <v>62</v>
       </c>
-      <c r="X9">
+      <c r="X9" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y9">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z9" t="s">
         <v>68</v>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="AR9">
         <f ca="1"/>
-        <v>244983366.60998237</v>
+        <v>665900380.87555802</v>
       </c>
       <c r="AS9" t="s">
         <v>82</v>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="L10">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M10" t="s">
         <v>56</v>
@@ -2656,13 +2656,13 @@
       <c r="W10" t="s">
         <v>62</v>
       </c>
-      <c r="X10">
+      <c r="X10" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y10">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z10" t="s">
         <v>68</v>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="AR10">
         <f ca="1"/>
-        <v>809086919.48819983</v>
+        <v>557604892.02107012</v>
       </c>
       <c r="AS10" t="s">
         <v>82</v>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="L11">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M11" t="s">
         <v>56</v>
@@ -2827,13 +2827,13 @@
       <c r="W11" t="s">
         <v>62</v>
       </c>
-      <c r="X11">
+      <c r="X11" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y11">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z11" t="s">
         <v>68</v>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="AR11">
         <f ca="1"/>
-        <v>491215807.22098196</v>
+        <v>401539222.41794133</v>
       </c>
       <c r="AS11" t="s">
         <v>82</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="L12">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M12" t="s">
         <v>56</v>
@@ -2998,13 +2998,13 @@
       <c r="W12" t="s">
         <v>62</v>
       </c>
-      <c r="X12">
+      <c r="X12" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y12">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z12" t="s">
         <v>68</v>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="AR12">
         <f ca="1"/>
-        <v>575273565.77730918</v>
+        <v>435720821.15358722</v>
       </c>
       <c r="AS12" t="s">
         <v>82</v>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="L13">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M13" t="s">
         <v>56</v>
@@ -3169,13 +3169,13 @@
       <c r="W13" t="s">
         <v>62</v>
       </c>
-      <c r="X13">
+      <c r="X13" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y13">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z13" t="s">
         <v>68</v>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AR13">
         <f ca="1"/>
-        <v>641166526.89329243</v>
+        <v>446462348.18625844</v>
       </c>
       <c r="AS13" t="s">
         <v>82</v>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="L14">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M14" t="s">
         <v>56</v>
@@ -3340,13 +3340,13 @@
       <c r="W14" t="s">
         <v>62</v>
       </c>
-      <c r="X14">
+      <c r="X14" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y14">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z14" t="s">
         <v>68</v>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="AR14">
         <f ca="1"/>
-        <v>564951556.47179794</v>
+        <v>573880861.22701013</v>
       </c>
       <c r="AS14" t="s">
         <v>82</v>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="L15">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M15" t="s">
         <v>56</v>
@@ -3511,13 +3511,13 @@
       <c r="W15" t="s">
         <v>62</v>
       </c>
-      <c r="X15">
+      <c r="X15" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y15">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z15" t="s">
         <v>68</v>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="AR15">
         <f ca="1"/>
-        <v>741238482.5467577</v>
+        <v>924238357.72275722</v>
       </c>
       <c r="AS15" t="s">
         <v>82</v>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="L16">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M16" t="s">
         <v>56</v>
@@ -3682,13 +3682,13 @@
       <c r="W16" t="s">
         <v>62</v>
       </c>
-      <c r="X16">
+      <c r="X16" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y16">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z16" t="s">
         <v>68</v>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="AR16">
         <f ca="1"/>
-        <v>978502636.12048495</v>
+        <v>298989757.24734187</v>
       </c>
       <c r="AS16" t="s">
         <v>82</v>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="L17">
         <f t="shared" ca="1" si="0"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="M17" t="s">
         <v>56</v>
@@ -3853,13 +3853,13 @@
       <c r="W17" t="s">
         <v>62</v>
       </c>
-      <c r="X17">
+      <c r="X17" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>45573</v>
+        <v>45576</v>
       </c>
       <c r="Y17">
         <f t="shared" ca="1" si="2"/>
-        <v>45624</v>
+        <v>45627</v>
       </c>
       <c r="Z17" t="s">
         <v>68</v>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="AR17">
         <f ca="1"/>
-        <v>995351386.61321211</v>
+        <v>202326851.60748303</v>
       </c>
       <c r="AS17" t="s">
         <v>82</v>

</xml_diff>